<commit_message>
docs(curadoria): aba 7 da V2 com o prazo do texto x tabela em casos reais (resumo anônimo)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/curadoria/hu14-pendencias-do-curador-v2.xlsx
+++ b/docs/curadoria/hu14-pendencias-do-curador-v2.xlsx
@@ -14,6 +14,7 @@
     <sheet name="4. Tabela de prazos" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="5. Calendário" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="6. Casos de teste" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="7. Texto x tabela" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -620,7 +621,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>1. Contradições · 2. Questões novas · 3. Fontes e vigência (regras) · 4. Tabela de prazos · 5. Calendário · 6. Casos de teste</t>
+          <t>1. Contradições · 2. Questões novas · 3. Fontes e vigência (regras) · 4. Tabela de prazos · 5. Calendário · 6. Casos de teste · 7. Texto x tabela (exemplos reais da contradição C02)</t>
         </is>
       </c>
     </row>
@@ -783,7 +784,7 @@
 3) Decisão aparentemente contrária a prazo legal expresso → mostrar os dois e exigir validação do advogado.
 4) Lei especial aplicável → prazo da lei especial.
 5) Sem identificar a regra → "a confirmar".
-Aprova assim? E o item "Prazo do ato judicial" passa de Dúvida para Aprovar ou Corrigir?</t>
+Veja os exemplos reais na aba 7. Aprova assim? E o item "Prazo do ato judicial" passa de Dúvida para Aprovar ou Corrigir?</t>
         </is>
       </c>
       <c r="F3" s="8" t="inlineStr"/>
@@ -8211,4 +8212,288 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="35" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>Situação encontrada</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
+          <t>Quantos (de 23 casos reais)</t>
+        </is>
+      </c>
+      <c r="C1" s="6" t="inlineStr">
+        <is>
+          <t>Exemplo (resumido, sem dados do processo)</t>
+        </is>
+      </c>
+      <c r="D1" s="6" t="inlineStr">
+        <is>
+          <t>Prazo no texto</t>
+        </is>
+      </c>
+      <c r="E1" s="6" t="inlineStr">
+        <is>
+          <t>Prazo na tabela V1</t>
+        </is>
+      </c>
+      <c r="F1" s="6" t="inlineStr">
+        <is>
+          <t>Qual deve valer? (curadora)</t>
+        </is>
+      </c>
+      <c r="G1" s="6" t="inlineStr">
+        <is>
+          <t>Fundamento (curadora)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="9" t="inlineStr">
+        <is>
+          <t>Fonte: 23 publicações reais do DJEN com prazo citado no texto, capturadas no ambiente de testes. Os casos completos (processo, trecho e sugestão de ato) estão na planilha CONFIDENCIAL hu14-texto-x-tabela-casos-reais, entregue à parte e fora do repositório.</t>
+        </is>
+      </c>
+      <c r="B2" s="10" t="n"/>
+      <c r="C2" s="10" t="n"/>
+      <c r="D2" s="10" t="n"/>
+      <c r="E2" s="10" t="n"/>
+      <c r="F2" s="10" t="n"/>
+      <c r="G2" s="11" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="9" t="inlineStr">
+        <is>
+          <t>Igual à tabela</t>
+        </is>
+      </c>
+      <c r="B3" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="C3" s="9" t="inlineStr">
+        <is>
+          <t>Especificação de provas em 5 dias; contestação cível em 15 dias úteis.</t>
+        </is>
+      </c>
+      <c r="D3" s="9" t="inlineStr">
+        <is>
+          <t>5 / 15 dias</t>
+        </is>
+      </c>
+      <c r="E3" s="9" t="inlineStr">
+        <is>
+          <t>5 / 15 dias úteis (linhas 5 e 2)</t>
+        </is>
+      </c>
+      <c r="F3" s="8" t="inlineStr"/>
+      <c r="G3" s="8" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>Juiz fixou prazo maior que o genérico (lei omissa?)</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>Manifestar-se sobre decisão, promover o andamento, juntar documento, recolher custas complementares, requerer após a baixa dos autos: todos em 15 dias.</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>15 dias</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>5 dias úteis (linha 12, CPC, art. 218, §3º)</t>
+        </is>
+      </c>
+      <c r="F4" s="8" t="inlineStr"/>
+      <c r="G4" s="8" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>Juiz fixou prazo onde a tabela não prevê prazo numérico</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>Juizado especial: contestar em 15 dias.</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>15 dias</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>Linha 90: sem prazo (contestação na audiência)</t>
+        </is>
+      </c>
+      <c r="F5" s="8" t="inlineStr"/>
+      <c r="G5" s="8" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>Tabela remete ao juiz</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>Juizado: juntar certidões em 5 dias.</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>5 dias</t>
+        </is>
+      </c>
+      <c r="E6" s="9" t="inlineStr">
+        <is>
+          <t>Linha 96: fixado pelo juízo</t>
+        </is>
+      </c>
+      <c r="F6" s="8" t="inlineStr"/>
+      <c r="G6" s="8" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>Prazo contado para trás a partir da audiência</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>Informar desinteresse na conciliação até 10 dias antes; apresentar rol de testemunhas até 5 dias úteis antes (trabalhista).</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>10 dias / 5 dias úteis</t>
+        </is>
+      </c>
+      <c r="E7" s="9" t="inlineStr">
+        <is>
+          <t>Sem linha na tabela</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="inlineStr"/>
+      <c r="G7" s="8" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>Prazo para terceiro, não para a parte</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>Perito: informar impedimento ou suspeição em 5 dias.</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>5 dias</t>
+        </is>
+      </c>
+      <c r="E8" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F8" s="8" t="inlineStr"/>
+      <c r="G8" s="8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>Não é prazo processual (a equipe corrige a leitura)</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="n">
+        <v>7</v>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>Cláusula penal de 3 meses de aluguel; restituição em até 12 meses; validade de documento de 120 dias.</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E9" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr"/>
+      <c r="G9" s="8" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>Pergunta: nas linhas em vermelho, o sistema deve sugerir o prazo do juiz (texto) ou o da tabela? Quando a lei for omissa (CPC, art. 218, §1º), confirma que vale o do juiz? E nos prazos contados para trás a partir da audiência, o sistema deve calcular (com regra própria) ou deixar "a confirmar"?</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="n"/>
+      <c r="C10" s="10" t="n"/>
+      <c r="D10" s="10" t="n"/>
+      <c r="E10" s="10" t="n"/>
+      <c r="F10" s="10" t="n"/>
+      <c r="G10" s="11" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A10:G10"/>
+  </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="F3:F9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Texto (prazo do juiz),Tabela (prazo legal),A confirmar,Não é prazo da parte"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>